<commit_message>
feat: Etapa 06 - MCP próprio (leitura e escrita com confirmação humana), tokens e testes com cliente MCP oficial
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q12tXbef8ejTamLrPrERvB
</commit_message>
<xml_diff>
--- a/docs/etapa-05/amostras/relatorio-executivo.xlsx
+++ b/docs/etapa-05/amostras/relatorio-executivo.xlsx
@@ -735,7 +735,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4">
-        <v>46306.634447696764</v>
+        <v>46306.640021087966</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>46306.634431597224</v>
+        <v>46306.64000461806</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1023,7 +1023,7 @@
         <v>46306</v>
       </c>
       <c r="R2" s="4">
-        <v>46306.634431597224</v>
+        <v>46306.64000461806</v>
       </c>
       <c r="S2" s="12" t="s">
         <v>40</v>
@@ -1080,7 +1080,7 @@
         <v>46306</v>
       </c>
       <c r="R3" s="4">
-        <v>46306.634431597224</v>
+        <v>46306.64000461806</v>
       </c>
       <c r="S3" s="12" t="s">
         <v>40</v>
@@ -1135,7 +1135,7 @@
         <v>46306</v>
       </c>
       <c r="R4" s="4">
-        <v>46306.634431597224</v>
+        <v>46306.64000461806</v>
       </c>
       <c r="S4" s="12" t="s">
         <v>40</v>
@@ -1192,7 +1192,7 @@
         <v>46306</v>
       </c>
       <c r="R5" s="4">
-        <v>46306.634431597224</v>
+        <v>46306.64000461806</v>
       </c>
       <c r="S5" s="12" t="s">
         <v>40</v>
@@ -1233,7 +1233,7 @@
         <v>46306</v>
       </c>
       <c r="R6" s="4">
-        <v>46306.634431597224</v>
+        <v>46306.64000461806</v>
       </c>
       <c r="S6" s="12" t="s">
         <v>40</v>
@@ -1272,7 +1272,7 @@
         <v>46306</v>
       </c>
       <c r="R7" s="4">
-        <v>46306.634431597224</v>
+        <v>46306.64000461806</v>
       </c>
       <c r="S7" s="12" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
docs: relatório final, saídas reais de testes/backup e prints da Etapa 07
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q12tXbef8ejTamLrPrERvB
</commit_message>
<xml_diff>
--- a/docs/etapa-05/amostras/relatorio-executivo.xlsx
+++ b/docs/etapa-05/amostras/relatorio-executivo.xlsx
@@ -735,7 +735,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4">
-        <v>46306.640021087966</v>
+        <v>46306.64606237269</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>46306.64000461806</v>
+        <v>46306.64604525463</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1023,7 +1023,7 @@
         <v>46306</v>
       </c>
       <c r="R2" s="4">
-        <v>46306.64000461806</v>
+        <v>46306.64604525463</v>
       </c>
       <c r="S2" s="12" t="s">
         <v>40</v>
@@ -1080,7 +1080,7 @@
         <v>46306</v>
       </c>
       <c r="R3" s="4">
-        <v>46306.64000461806</v>
+        <v>46306.64604525463</v>
       </c>
       <c r="S3" s="12" t="s">
         <v>40</v>
@@ -1135,7 +1135,7 @@
         <v>46306</v>
       </c>
       <c r="R4" s="4">
-        <v>46306.64000461806</v>
+        <v>46306.64604525463</v>
       </c>
       <c r="S4" s="12" t="s">
         <v>40</v>
@@ -1192,7 +1192,7 @@
         <v>46306</v>
       </c>
       <c r="R5" s="4">
-        <v>46306.64000461806</v>
+        <v>46306.64604525463</v>
       </c>
       <c r="S5" s="12" t="s">
         <v>40</v>
@@ -1233,7 +1233,7 @@
         <v>46306</v>
       </c>
       <c r="R6" s="4">
-        <v>46306.64000461806</v>
+        <v>46306.64604525463</v>
       </c>
       <c r="S6" s="12" t="s">
         <v>40</v>
@@ -1272,7 +1272,7 @@
         <v>46306</v>
       </c>
       <c r="R7" s="4">
-        <v>46306.64000461806</v>
+        <v>46306.64604525463</v>
       </c>
       <c r="S7" s="12" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
feat: acesso restrito por conta de anúncios para cada membro (telas, relatórios, operações, MCP)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q12tXbef8ejTamLrPrERvB
</commit_message>
<xml_diff>
--- a/docs/etapa-05/amostras/relatorio-executivo.xlsx
+++ b/docs/etapa-05/amostras/relatorio-executivo.xlsx
@@ -735,7 +735,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4">
-        <v>46306.64606237269</v>
+        <v>46306.65119430555</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>46306.64604525463</v>
+        <v>46306.65117971065</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -765,13 +765,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="7">
-        <v>12759.339999999997</v>
+        <v>12759.339999999998</v>
       </c>
       <c r="C11" s="7">
         <v>12785.670000000004</v>
       </c>
       <c r="D11" s="8">
-        <v>-0.002059336741837322</v>
+        <v>-0.00205933674183718</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -821,13 +821,13 @@
         <v>20</v>
       </c>
       <c r="B15" s="7">
-        <v>6.6351222048881935</v>
+        <v>6.635122204888194</v>
       </c>
       <c r="C15" s="7">
         <v>6.739942013705853</v>
       </c>
       <c r="D15" s="8">
-        <v>-0.015552034216986744</v>
+        <v>-0.01555203421698661</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -849,13 +849,13 @@
         <v>22</v>
       </c>
       <c r="B17" s="7">
-        <v>0.7570511451287526</v>
+        <v>0.7570511451287527</v>
       </c>
       <c r="C17" s="7">
         <v>0.7465212821860223</v>
       </c>
       <c r="D17" s="8">
-        <v>0.014105241463305522</v>
+        <v>0.014105241463305671</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -863,13 +863,13 @@
         <v>23</v>
       </c>
       <c r="B18" s="7">
-        <v>14.07056156133968</v>
+        <v>14.070561561339682</v>
       </c>
       <c r="C18" s="7">
         <v>13.89434116454233</v>
       </c>
       <c r="D18" s="8">
-        <v>0.012682889725426865</v>
+        <v>0.012682889725426992</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1023,7 +1023,7 @@
         <v>46306</v>
       </c>
       <c r="R2" s="4">
-        <v>46306.64604525463</v>
+        <v>46306.65117971065</v>
       </c>
       <c r="S2" s="12" t="s">
         <v>40</v>
@@ -1080,7 +1080,7 @@
         <v>46306</v>
       </c>
       <c r="R3" s="4">
-        <v>46306.64604525463</v>
+        <v>46306.65117971065</v>
       </c>
       <c r="S3" s="12" t="s">
         <v>40</v>
@@ -1135,7 +1135,7 @@
         <v>46306</v>
       </c>
       <c r="R4" s="4">
-        <v>46306.64604525463</v>
+        <v>46306.65117971065</v>
       </c>
       <c r="S4" s="12" t="s">
         <v>40</v>
@@ -1192,7 +1192,7 @@
         <v>46306</v>
       </c>
       <c r="R5" s="4">
-        <v>46306.64604525463</v>
+        <v>46306.65117971065</v>
       </c>
       <c r="S5" s="12" t="s">
         <v>40</v>
@@ -1233,7 +1233,7 @@
         <v>46306</v>
       </c>
       <c r="R6" s="4">
-        <v>46306.64604525463</v>
+        <v>46306.65117971065</v>
       </c>
       <c r="S6" s="12" t="s">
         <v>40</v>
@@ -1272,7 +1272,7 @@
         <v>46306</v>
       </c>
       <c r="R7" s="4">
-        <v>46306.64604525463</v>
+        <v>46306.65117971065</v>
       </c>
       <c r="S7" s="12" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
feat: logo da empresa nos relatórios (PDF, XLSX e tela) com upload seguro e verificação
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q12tXbef8ejTamLrPrERvB
</commit_message>
<xml_diff>
--- a/docs/etapa-05/amostras/relatorio-executivo.xlsx
+++ b/docs/etapa-05/amostras/relatorio-executivo.xlsx
@@ -735,7 +735,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4">
-        <v>46306.65119430555</v>
+        <v>46306.65585435185</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>46306.65117971065</v>
+        <v>46306.65584274306</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1023,7 +1023,7 @@
         <v>46306</v>
       </c>
       <c r="R2" s="4">
-        <v>46306.65117971065</v>
+        <v>46306.65584274306</v>
       </c>
       <c r="S2" s="12" t="s">
         <v>40</v>
@@ -1080,7 +1080,7 @@
         <v>46306</v>
       </c>
       <c r="R3" s="4">
-        <v>46306.65117971065</v>
+        <v>46306.65584274306</v>
       </c>
       <c r="S3" s="12" t="s">
         <v>40</v>
@@ -1135,7 +1135,7 @@
         <v>46306</v>
       </c>
       <c r="R4" s="4">
-        <v>46306.65117971065</v>
+        <v>46306.65584274306</v>
       </c>
       <c r="S4" s="12" t="s">
         <v>40</v>
@@ -1192,7 +1192,7 @@
         <v>46306</v>
       </c>
       <c r="R5" s="4">
-        <v>46306.65117971065</v>
+        <v>46306.65584274306</v>
       </c>
       <c r="S5" s="12" t="s">
         <v>40</v>
@@ -1233,7 +1233,7 @@
         <v>46306</v>
       </c>
       <c r="R6" s="4">
-        <v>46306.65117971065</v>
+        <v>46306.65584274306</v>
       </c>
       <c r="S6" s="12" t="s">
         <v>40</v>
@@ -1272,7 +1272,7 @@
         <v>46306</v>
       </c>
       <c r="R7" s="4">
-        <v>46306.65117971065</v>
+        <v>46306.65584274306</v>
       </c>
       <c r="S7" s="12" t="s">
         <v>40</v>
@@ -1419,7 +1419,7 @@
         <v>46283</v>
       </c>
       <c r="B8" s="7">
-        <v>436.22999999999996</v>
+        <v>436.23</v>
       </c>
       <c r="C8" s="9">
         <v>30139</v>
@@ -1521,7 +1521,7 @@
         <v>46289</v>
       </c>
       <c r="B14" s="7">
-        <v>413.27000000000004</v>
+        <v>413.27</v>
       </c>
       <c r="C14" s="9">
         <v>29504</v>
@@ -1538,7 +1538,7 @@
         <v>46290</v>
       </c>
       <c r="B15" s="7">
-        <v>452.15999999999997</v>
+        <v>452.16</v>
       </c>
       <c r="C15" s="9">
         <v>31515</v>
@@ -1555,7 +1555,7 @@
         <v>46291</v>
       </c>
       <c r="B16" s="7">
-        <v>479.18</v>
+        <v>479.17999999999995</v>
       </c>
       <c r="C16" s="9">
         <v>35008</v>
@@ -1810,7 +1810,7 @@
         <v>46306</v>
       </c>
       <c r="B31" s="7">
-        <v>425.20000000000005</v>
+        <v>425.2</v>
       </c>
       <c r="C31" s="9">
         <v>31363</v>

</xml_diff>

<commit_message>
feat(v2): Etapa 02 - fundação (erro/404/carregamento, CSP com nonce, cron seguro, ESLint, log de erros, skip link)
</commit_message>
<xml_diff>
--- a/docs/etapa-05/amostras/relatorio-executivo.xlsx
+++ b/docs/etapa-05/amostras/relatorio-executivo.xlsx
@@ -735,7 +735,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4">
-        <v>46306.65585435185</v>
+        <v>46306.924109942134</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>46306.65584274306</v>
+        <v>46306.92409554398</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -768,10 +768,10 @@
         <v>12759.339999999998</v>
       </c>
       <c r="C11" s="7">
-        <v>12785.670000000004</v>
+        <v>12785.669999999996</v>
       </c>
       <c r="D11" s="8">
-        <v>-0.00205933674183718</v>
+        <v>-0.0020593367418366123</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -824,10 +824,10 @@
         <v>6.635122204888194</v>
       </c>
       <c r="C15" s="7">
-        <v>6.739942013705853</v>
+        <v>6.73994201370585</v>
       </c>
       <c r="D15" s="8">
-        <v>-0.01555203421698661</v>
+        <v>-0.015552034216986093</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -852,10 +852,10 @@
         <v>0.7570511451287527</v>
       </c>
       <c r="C17" s="7">
-        <v>0.7465212821860223</v>
+        <v>0.7465212821860219</v>
       </c>
       <c r="D17" s="8">
-        <v>0.014105241463305671</v>
+        <v>0.014105241463306273</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -866,10 +866,10 @@
         <v>14.070561561339682</v>
       </c>
       <c r="C18" s="7">
-        <v>13.89434116454233</v>
+        <v>13.894341164542322</v>
       </c>
       <c r="D18" s="8">
-        <v>0.012682889725426992</v>
+        <v>0.012682889725427643</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1023,7 +1023,7 @@
         <v>46306</v>
       </c>
       <c r="R2" s="4">
-        <v>46306.65584274306</v>
+        <v>46306.92409554398</v>
       </c>
       <c r="S2" s="12" t="s">
         <v>40</v>
@@ -1080,7 +1080,7 @@
         <v>46306</v>
       </c>
       <c r="R3" s="4">
-        <v>46306.65584274306</v>
+        <v>46306.92409554398</v>
       </c>
       <c r="S3" s="12" t="s">
         <v>40</v>
@@ -1135,7 +1135,7 @@
         <v>46306</v>
       </c>
       <c r="R4" s="4">
-        <v>46306.65584274306</v>
+        <v>46306.92409554398</v>
       </c>
       <c r="S4" s="12" t="s">
         <v>40</v>
@@ -1192,7 +1192,7 @@
         <v>46306</v>
       </c>
       <c r="R5" s="4">
-        <v>46306.65584274306</v>
+        <v>46306.92409554398</v>
       </c>
       <c r="S5" s="12" t="s">
         <v>40</v>
@@ -1233,7 +1233,7 @@
         <v>46306</v>
       </c>
       <c r="R6" s="4">
-        <v>46306.65584274306</v>
+        <v>46306.92409554398</v>
       </c>
       <c r="S6" s="12" t="s">
         <v>40</v>
@@ -1272,7 +1272,7 @@
         <v>46306</v>
       </c>
       <c r="R7" s="4">
-        <v>46306.65584274306</v>
+        <v>46306.92409554398</v>
       </c>
       <c r="S7" s="12" t="s">
         <v>40</v>
@@ -1419,7 +1419,7 @@
         <v>46283</v>
       </c>
       <c r="B8" s="7">
-        <v>436.23</v>
+        <v>436.22999999999996</v>
       </c>
       <c r="C8" s="9">
         <v>30139</v>
@@ -1521,7 +1521,7 @@
         <v>46289</v>
       </c>
       <c r="B14" s="7">
-        <v>413.27</v>
+        <v>413.27000000000004</v>
       </c>
       <c r="C14" s="9">
         <v>29504</v>
@@ -1538,7 +1538,7 @@
         <v>46290</v>
       </c>
       <c r="B15" s="7">
-        <v>452.16</v>
+        <v>452.15999999999997</v>
       </c>
       <c r="C15" s="9">
         <v>31515</v>
@@ -1555,7 +1555,7 @@
         <v>46291</v>
       </c>
       <c r="B16" s="7">
-        <v>479.17999999999995</v>
+        <v>479.18</v>
       </c>
       <c r="C16" s="9">
         <v>35008</v>
@@ -1810,7 +1810,7 @@
         <v>46306</v>
       </c>
       <c r="B31" s="7">
-        <v>425.2</v>
+        <v>425.20000000000005</v>
       </c>
       <c r="C31" s="9">
         <v>31363</v>

</xml_diff>

<commit_message>
Etapa 03: E2E de gestão, correção de menu lateral, relatório e prints
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q12tXbef8ejTamLrPrERvB
</commit_message>
<xml_diff>
--- a/docs/etapa-05/amostras/relatorio-executivo.xlsx
+++ b/docs/etapa-05/amostras/relatorio-executivo.xlsx
@@ -735,7 +735,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4">
-        <v>46306.924109942134</v>
+        <v>46306.94012126158</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>46306.92409554398</v>
+        <v>46306.94010546296</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -765,13 +765,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="7">
-        <v>12759.339999999998</v>
+        <v>12759.34</v>
       </c>
       <c r="C11" s="7">
         <v>12785.669999999996</v>
       </c>
       <c r="D11" s="8">
-        <v>-0.0020593367418366123</v>
+        <v>-0.0020593367418364696</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -821,13 +821,13 @@
         <v>20</v>
       </c>
       <c r="B15" s="7">
-        <v>6.635122204888194</v>
+        <v>6.635122204888195</v>
       </c>
       <c r="C15" s="7">
         <v>6.73994201370585</v>
       </c>
       <c r="D15" s="8">
-        <v>-0.015552034216986093</v>
+        <v>-0.01555203421698596</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -849,13 +849,13 @@
         <v>22</v>
       </c>
       <c r="B17" s="7">
-        <v>0.7570511451287527</v>
+        <v>0.7570511451287528</v>
       </c>
       <c r="C17" s="7">
         <v>0.7465212821860219</v>
       </c>
       <c r="D17" s="8">
-        <v>0.014105241463306273</v>
+        <v>0.014105241463306422</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -863,13 +863,13 @@
         <v>23</v>
       </c>
       <c r="B18" s="7">
-        <v>14.070561561339682</v>
+        <v>14.070561561339684</v>
       </c>
       <c r="C18" s="7">
         <v>13.894341164542322</v>
       </c>
       <c r="D18" s="8">
-        <v>0.012682889725427643</v>
+        <v>0.01268288972542777</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1023,7 +1023,7 @@
         <v>46306</v>
       </c>
       <c r="R2" s="4">
-        <v>46306.92409554398</v>
+        <v>46306.94010546296</v>
       </c>
       <c r="S2" s="12" t="s">
         <v>40</v>
@@ -1080,7 +1080,7 @@
         <v>46306</v>
       </c>
       <c r="R3" s="4">
-        <v>46306.92409554398</v>
+        <v>46306.94010546296</v>
       </c>
       <c r="S3" s="12" t="s">
         <v>40</v>
@@ -1135,7 +1135,7 @@
         <v>46306</v>
       </c>
       <c r="R4" s="4">
-        <v>46306.92409554398</v>
+        <v>46306.94010546296</v>
       </c>
       <c r="S4" s="12" t="s">
         <v>40</v>
@@ -1192,7 +1192,7 @@
         <v>46306</v>
       </c>
       <c r="R5" s="4">
-        <v>46306.92409554398</v>
+        <v>46306.94010546296</v>
       </c>
       <c r="S5" s="12" t="s">
         <v>40</v>
@@ -1233,7 +1233,7 @@
         <v>46306</v>
       </c>
       <c r="R6" s="4">
-        <v>46306.92409554398</v>
+        <v>46306.94010546296</v>
       </c>
       <c r="S6" s="12" t="s">
         <v>40</v>
@@ -1272,7 +1272,7 @@
         <v>46306</v>
       </c>
       <c r="R7" s="4">
-        <v>46306.92409554398</v>
+        <v>46306.94010546296</v>
       </c>
       <c r="S7" s="12" t="s">
         <v>40</v>
@@ -1317,7 +1317,7 @@
         <v>46277</v>
       </c>
       <c r="B2" s="7">
-        <v>419.66999999999996</v>
+        <v>419.67</v>
       </c>
       <c r="C2" s="9">
         <v>29433</v>
@@ -1334,7 +1334,7 @@
         <v>46278</v>
       </c>
       <c r="B3" s="7">
-        <v>456.79</v>
+        <v>456.78999999999996</v>
       </c>
       <c r="C3" s="9">
         <v>31758</v>
@@ -1436,7 +1436,7 @@
         <v>46284</v>
       </c>
       <c r="B9" s="7">
-        <v>366.94000000000005</v>
+        <v>366.94</v>
       </c>
       <c r="C9" s="9">
         <v>25222</v>
@@ -1453,7 +1453,7 @@
         <v>46285</v>
       </c>
       <c r="B10" s="7">
-        <v>428.45000000000005</v>
+        <v>428.45</v>
       </c>
       <c r="C10" s="9">
         <v>29750</v>
@@ -1470,7 +1470,7 @@
         <v>46286</v>
       </c>
       <c r="B11" s="7">
-        <v>417.24</v>
+        <v>417.23999999999995</v>
       </c>
       <c r="C11" s="9">
         <v>29817</v>
@@ -1555,7 +1555,7 @@
         <v>46291</v>
       </c>
       <c r="B16" s="7">
-        <v>479.18</v>
+        <v>479.18000000000006</v>
       </c>
       <c r="C16" s="9">
         <v>35008</v>
@@ -1589,7 +1589,7 @@
         <v>46293</v>
       </c>
       <c r="B18" s="7">
-        <v>448.43</v>
+        <v>448.42999999999995</v>
       </c>
       <c r="C18" s="9">
         <v>31119</v>
@@ -1691,7 +1691,7 @@
         <v>46299</v>
       </c>
       <c r="B24" s="7">
-        <v>402.28999999999996</v>
+        <v>402.29</v>
       </c>
       <c r="C24" s="9">
         <v>28262</v>
@@ -1776,7 +1776,7 @@
         <v>46304</v>
       </c>
       <c r="B29" s="7">
-        <v>435.97999999999996</v>
+        <v>435.98</v>
       </c>
       <c r="C29" s="9">
         <v>30656</v>
@@ -1793,7 +1793,7 @@
         <v>46305</v>
       </c>
       <c r="B30" s="7">
-        <v>436.49</v>
+        <v>436.48999999999995</v>
       </c>
       <c r="C30" s="9">
         <v>30474</v>
@@ -1810,7 +1810,7 @@
         <v>46306</v>
       </c>
       <c r="B31" s="7">
-        <v>425.20000000000005</v>
+        <v>425.2</v>
       </c>
       <c r="C31" s="9">
         <v>31363</v>

</xml_diff>

<commit_message>
Etapa 07: verificação final, prints finais, relatório e checklist de produção; correções de acessibilidade
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q12tXbef8ejTamLrPrERvB
</commit_message>
<xml_diff>
--- a/docs/etapa-05/amostras/relatorio-executivo.xlsx
+++ b/docs/etapa-05/amostras/relatorio-executivo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
   <si>
     <t>AdsPilot — Resumo executivo</t>
   </si>
@@ -89,6 +89,21 @@
   </si>
   <si>
     <t>ROAS</t>
+  </si>
+  <si>
+    <t>Leads</t>
+  </si>
+  <si>
+    <t>CPL (custo por lead)</t>
+  </si>
+  <si>
+    <t>Compras</t>
+  </si>
+  <si>
+    <t>CPA (custo por compra)</t>
+  </si>
+  <si>
+    <t>Taxa de conversão (resultados ÷ cliques)</t>
   </si>
   <si>
     <t>Campanha</t>
@@ -680,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -735,7 +750,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4">
-        <v>46306.94012126158</v>
+        <v>46306.957747673616</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +758,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>46306.94010546296</v>
+        <v>46306.95773425926</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -765,13 +780,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="7">
-        <v>12759.34</v>
+        <v>12759.339999999997</v>
       </c>
       <c r="C11" s="7">
-        <v>12785.669999999996</v>
+        <v>12785.670000000004</v>
       </c>
       <c r="D11" s="8">
-        <v>-0.0020593367418364696</v>
+        <v>-0.002059336741837322</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -821,13 +836,13 @@
         <v>20</v>
       </c>
       <c r="B15" s="7">
-        <v>6.635122204888195</v>
+        <v>6.6351222048881935</v>
       </c>
       <c r="C15" s="7">
-        <v>6.73994201370585</v>
+        <v>6.739942013705853</v>
       </c>
       <c r="D15" s="8">
-        <v>-0.01555203421698596</v>
+        <v>-0.015552034216986744</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -849,13 +864,13 @@
         <v>22</v>
       </c>
       <c r="B17" s="7">
-        <v>0.7570511451287528</v>
+        <v>0.7570511451287526</v>
       </c>
       <c r="C17" s="7">
-        <v>0.7465212821860219</v>
+        <v>0.7465212821860223</v>
       </c>
       <c r="D17" s="8">
-        <v>0.014105241463306422</v>
+        <v>0.014105241463305522</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -863,13 +878,13 @@
         <v>23</v>
       </c>
       <c r="B18" s="7">
-        <v>14.070561561339684</v>
+        <v>14.07056156133968</v>
       </c>
       <c r="C18" s="7">
-        <v>13.894341164542322</v>
+        <v>13.89434116454233</v>
       </c>
       <c r="D18" s="8">
-        <v>0.01268288972542777</v>
+        <v>0.012682889725426865</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -884,6 +899,76 @@
       </c>
       <c r="D19" s="8">
         <v>-5.068916758014455e-7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="9">
+        <v>310</v>
+      </c>
+      <c r="C20" s="9">
+        <v>312</v>
+      </c>
+      <c r="D20" s="8">
+        <v>-0.00641025641025641</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="7">
+        <v>18.571999999999996</v>
+      </c>
+      <c r="C21" s="7">
+        <v>18.554102564102557</v>
+      </c>
+      <c r="D21" s="8">
+        <v>0.0009646080070757828</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="9">
+        <v>366</v>
+      </c>
+      <c r="C22" s="9">
+        <v>369</v>
+      </c>
+      <c r="D22" s="8">
+        <v>-0.008130081300813009</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="7">
+        <v>15.387295081967215</v>
+      </c>
+      <c r="C23" s="7">
+        <v>15.341300813008132</v>
+      </c>
+      <c r="D23" s="8">
+        <v>0.002998068385445099</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="10">
+        <v>0.11409754360982555</v>
+      </c>
+      <c r="C24" s="10">
+        <v>0.1107607870613651</v>
+      </c>
+      <c r="D24" s="8">
+        <v>0.030125793044534624</v>
       </c>
     </row>
   </sheetData>
@@ -913,7 +998,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:19" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B1" s="15" t="s">
         <v>6</v>
@@ -922,13 +1007,13 @@
         <v>4</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="G1" s="17" t="s">
         <v>17</v>
@@ -943,7 +1028,7 @@
         <v>20</v>
       </c>
       <c r="K1" s="18" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="L1" s="16" t="s">
         <v>22</v>
@@ -955,36 +1040,36 @@
         <v>24</v>
       </c>
       <c r="O1" s="15" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="P1" s="20" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="Q1" s="20" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="R1" s="21" t="s">
         <v>11</v>
       </c>
       <c r="S1" s="15" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F2" s="7">
         <v>5631.750000000001</v>
@@ -1014,7 +1099,7 @@
         <v>4.199998224352998</v>
       </c>
       <c r="O2" s="12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="P2" s="13">
         <v>46277</v>
@@ -1023,27 +1108,27 @@
         <v>46306</v>
       </c>
       <c r="R2" s="4">
-        <v>46306.94010546296</v>
+        <v>46306.95773425926</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>36</v>
-      </c>
       <c r="D3" s="12" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F3" s="7">
         <v>3414.4700000000003</v>
@@ -1071,7 +1156,7 @@
       </c>
       <c r="N3" s="11"/>
       <c r="O3" s="12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="P3" s="13">
         <v>46277</v>
@@ -1080,25 +1165,25 @@
         <v>46306</v>
       </c>
       <c r="R3" s="4">
-        <v>46306.94010546296</v>
+        <v>46306.95773425926</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F4" s="7">
         <v>2342.8500000000004</v>
@@ -1126,7 +1211,7 @@
       </c>
       <c r="N4" s="11"/>
       <c r="O4" s="12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="P4" s="13">
         <v>46277</v>
@@ -1135,27 +1220,27 @@
         <v>46306</v>
       </c>
       <c r="R4" s="4">
-        <v>46306.94010546296</v>
+        <v>46306.95773425926</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F5" s="7">
         <v>1370.27</v>
@@ -1183,7 +1268,7 @@
       </c>
       <c r="N5" s="11"/>
       <c r="O5" s="12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="P5" s="13">
         <v>46277</v>
@@ -1192,27 +1277,27 @@
         <v>46306</v>
       </c>
       <c r="R5" s="4">
-        <v>46306.94010546296</v>
+        <v>46306.95773425926</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="9"/>
@@ -1224,7 +1309,7 @@
       <c r="M6" s="7"/>
       <c r="N6" s="11"/>
       <c r="O6" s="12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="P6" s="13">
         <v>46277</v>
@@ -1233,25 +1318,25 @@
         <v>46306</v>
       </c>
       <c r="R6" s="4">
-        <v>46306.94010546296</v>
+        <v>46306.95773425926</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="9"/>
@@ -1263,7 +1348,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="11"/>
       <c r="O7" s="12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="P7" s="13">
         <v>46277</v>
@@ -1272,10 +1357,10 @@
         <v>46306</v>
       </c>
       <c r="R7" s="4">
-        <v>46306.94010546296</v>
+        <v>46306.95773425926</v>
       </c>
       <c r="S7" s="12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1297,10 +1382,10 @@
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C1" s="24" t="s">
         <v>17</v>
@@ -1317,7 +1402,7 @@
         <v>46277</v>
       </c>
       <c r="B2" s="7">
-        <v>419.67</v>
+        <v>419.66999999999996</v>
       </c>
       <c r="C2" s="9">
         <v>29433</v>
@@ -1334,7 +1419,7 @@
         <v>46278</v>
       </c>
       <c r="B3" s="7">
-        <v>456.78999999999996</v>
+        <v>456.79</v>
       </c>
       <c r="C3" s="9">
         <v>31758</v>
@@ -1419,7 +1504,7 @@
         <v>46283</v>
       </c>
       <c r="B8" s="7">
-        <v>436.22999999999996</v>
+        <v>436.23</v>
       </c>
       <c r="C8" s="9">
         <v>30139</v>
@@ -1436,7 +1521,7 @@
         <v>46284</v>
       </c>
       <c r="B9" s="7">
-        <v>366.94</v>
+        <v>366.93999999999994</v>
       </c>
       <c r="C9" s="9">
         <v>25222</v>
@@ -1453,7 +1538,7 @@
         <v>46285</v>
       </c>
       <c r="B10" s="7">
-        <v>428.45</v>
+        <v>428.45000000000005</v>
       </c>
       <c r="C10" s="9">
         <v>29750</v>
@@ -1470,7 +1555,7 @@
         <v>46286</v>
       </c>
       <c r="B11" s="7">
-        <v>417.23999999999995</v>
+        <v>417.24</v>
       </c>
       <c r="C11" s="9">
         <v>29817</v>
@@ -1521,7 +1606,7 @@
         <v>46289</v>
       </c>
       <c r="B14" s="7">
-        <v>413.27000000000004</v>
+        <v>413.27</v>
       </c>
       <c r="C14" s="9">
         <v>29504</v>
@@ -1538,7 +1623,7 @@
         <v>46290</v>
       </c>
       <c r="B15" s="7">
-        <v>452.15999999999997</v>
+        <v>452.16</v>
       </c>
       <c r="C15" s="9">
         <v>31515</v>
@@ -1555,7 +1640,7 @@
         <v>46291</v>
       </c>
       <c r="B16" s="7">
-        <v>479.18000000000006</v>
+        <v>479.17999999999995</v>
       </c>
       <c r="C16" s="9">
         <v>35008</v>
@@ -1589,7 +1674,7 @@
         <v>46293</v>
       </c>
       <c r="B18" s="7">
-        <v>448.42999999999995</v>
+        <v>448.43</v>
       </c>
       <c r="C18" s="9">
         <v>31119</v>
@@ -1691,7 +1776,7 @@
         <v>46299</v>
       </c>
       <c r="B24" s="7">
-        <v>402.29</v>
+        <v>402.28999999999996</v>
       </c>
       <c r="C24" s="9">
         <v>28262</v>
@@ -1776,7 +1861,7 @@
         <v>46304</v>
       </c>
       <c r="B29" s="7">
-        <v>435.98</v>
+        <v>435.97999999999996</v>
       </c>
       <c r="C29" s="9">
         <v>30656</v>
@@ -1793,7 +1878,7 @@
         <v>46305</v>
       </c>
       <c r="B30" s="7">
-        <v>436.48999999999995</v>
+        <v>436.49</v>
       </c>
       <c r="C30" s="9">
         <v>30474</v>
@@ -1839,122 +1924,122 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>